<commit_message>
pd-cli@v1.0.3: Enable multiple value insert or update in FLS and Apex Secuerity
</commit_message>
<xml_diff>
--- a/post-deploy-tasks.xlsx
+++ b/post-deploy-tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Subhadeep_Sarkar\Desktop\SkillSet\Node js\Salesforce PD Task Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB94586-4B7B-4D3F-B32B-7C803E2DF642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B279BE-19E4-403B-BEFE-46E892F29822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>Task #</t>
   </si>
@@ -65,9 +65,6 @@
     <t>FLS</t>
   </si>
   <si>
-    <t>Custom: Sales Profile</t>
-  </si>
-  <si>
     <t>Account</t>
   </si>
   <si>
@@ -98,9 +95,6 @@
     <t>ApexAccess</t>
   </si>
   <si>
-    <t>Standard User</t>
-  </si>
-  <si>
     <t>OpportunityClass</t>
   </si>
   <si>
@@ -113,9 +107,6 @@
     <t>Test PD Account</t>
   </si>
   <si>
-    <t>{"Industry":"Technology","Phone":"1234567890"}</t>
-  </si>
-  <si>
     <t>Demo data</t>
   </si>
   <si>
@@ -144,6 +135,21 @@
   </si>
   <si>
     <t>Test LOV</t>
+  </si>
+  <si>
+    <t>Custom: Sales Profile,Custom: Support Profile,Custom: Marketing Profile</t>
+  </si>
+  <si>
+    <t>Standard User,Customer Community User,Customer Portal Manager Custom,Customer Portal Manager Standard</t>
+  </si>
+  <si>
+    <t>Operation</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>{"Id":"001WU00001rcIL8YAM","Industry":"Technology","Phone":"1234567890"}</t>
   </si>
 </sst>
 </file>
@@ -527,7 +533,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.109375" style="5" bestFit="1" customWidth="1"/>
@@ -540,12 +546,13 @@
     <col min="12" max="12" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="22.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -568,16 +575,16 @@
         <v>6</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>35</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>7</v>
@@ -589,16 +596,19 @@
         <v>9</v>
       </c>
       <c r="O1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="P1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="R1" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -606,19 +616,19 @@
         <v>13</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>18</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -629,11 +639,12 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-      <c r="Q2" s="3" t="s">
-        <v>19</v>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -641,19 +652,19 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>22</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -664,19 +675,20 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
-      <c r="Q3" s="3" t="s">
-        <v>23</v>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -687,24 +699,25 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="3" t="s">
-        <v>27</v>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -718,36 +731,39 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>31</v>
+        <v>42</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J6" s="1" t="b">
         <v>1</v>
@@ -755,8 +771,8 @@
       <c r="K6" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="Q6" s="1" t="s">
-        <v>40</v>
+      <c r="R6" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pd-cli@v1.0.3: Removed Name dependency & Improved excel sheet
</commit_message>
<xml_diff>
--- a/post-deploy-tasks.xlsx
+++ b/post-deploy-tasks.xlsx
@@ -1,27 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Subhadeep_Sarkar\Desktop\SkillSet\Node js\Salesforce PD Task Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B279BE-19E4-403B-BEFE-46E892F29822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{435D0842-CA1D-4FFA-A7C0-F3385D36D4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Input" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>Task #</t>
   </si>
@@ -53,9 +64,6 @@
     <t>SObject Type</t>
   </si>
   <si>
-    <t>Record Name</t>
-  </si>
-  <si>
     <t>Additional Fields (JSON)</t>
   </si>
   <si>
@@ -71,12 +79,6 @@
     <t>AnnualRevenue</t>
   </si>
   <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
     <t>For sales visibility</t>
   </si>
   <si>
@@ -104,9 +106,6 @@
     <t>Record</t>
   </si>
   <si>
-    <t>Test PD Account</t>
-  </si>
-  <si>
     <t>Demo data</t>
   </si>
   <si>
@@ -146,10 +145,13 @@
     <t>Operation</t>
   </si>
   <si>
+    <t>User_Story__c</t>
+  </si>
+  <si>
+    <t>{"Description__c":"Test description from PD Automation v2","Assigned_Developer__c":"a0FWU000008vPgD2AU","Id":"a0GWU00000LKx4f2AD"}</t>
+  </si>
+  <si>
     <t>update</t>
-  </si>
-  <si>
-    <t>{"Id":"001WU00001rcIL8YAM","Industry":"Technology","Phone":"1234567890"}</t>
   </si>
 </sst>
 </file>
@@ -205,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -219,20 +221,68 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="3" tint="0.59996337778862885"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="3" tint="0.39994506668294322"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="3" tint="0.39994506668294322"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.499984740745262"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor theme="3" tint="0.39994506668294322"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -530,105 +580,102 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="11" width="9.88671875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5546875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="22.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.88671875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="9.88671875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="17.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" style="8" customWidth="1"/>
+    <col min="14" max="14" width="15.109375" style="8" customWidth="1"/>
+    <col min="15" max="15" width="11.5546875" style="8" customWidth="1"/>
+    <col min="16" max="16" width="22.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.6640625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:17" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="L1" s="7" t="s">
+      <c r="H1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="N1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="P1" s="7" t="s">
+      <c r="O1" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="R1" s="7" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" s="1" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>17</v>
+      <c r="F2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="b">
+        <v>0</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -639,32 +686,31 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3" t="s">
-        <v>18</v>
+      <c r="Q2" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:18" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" s="1" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="F3" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -675,20 +721,19 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3" t="s">
-        <v>22</v>
+      <c r="Q3" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:18" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" s="1" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -699,25 +744,24 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>16</v>
+        <v>21</v>
+      </c>
+      <c r="M4" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3" t="s">
-        <v>25</v>
+      <c r="Q4" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:18" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" s="1" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -731,57 +775,86 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="P5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="Q5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="R5" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="1" t="b">
+      <c r="H6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="J6" s="8" t="b">
         <v>1</v>
       </c>
-      <c r="K6" s="1" t="b">
+      <c r="K6" s="8" t="b">
         <v>0</v>
       </c>
-      <c r="R6" s="1" t="s">
-        <v>37</v>
+      <c r="Q6" s="8" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C1:C1048576 F1:G1048576 L1:P1048576">
+    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
+      <formula>$B1="PicklistValue"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1:M1048576">
+    <cfRule type="expression" dxfId="2" priority="2" stopIfTrue="1">
+      <formula>$B1="Record"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:K1048576 N1:P1048576">
+    <cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
+      <formula>$B1="ApexAccess"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:P1048576">
+    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
+      <formula>$B1="FLS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Task Type" error="Please select a task type from the dropdown" promptTitle="Task Type" prompt="Select the type of task:_x000a_  - FLS: Field-Level Security_x000a_  - ApexAccess: Apex Class Access_x000a_  - PicklistValue: Add picklist values_x000a_  - Record: Create/Update records" sqref="B1:B1048576" xr:uid="{92766FC8-EFE2-4B5A-B064-D5326743F562}">
+      <formula1>"FLS,ApexAccess,Record,PicklistValue"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J1:K1048576 M1:M1048576 F1:G1048576" xr:uid="{A56FC731-9A7C-45FA-88CF-83E189D8CB59}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O1:O1048576" xr:uid="{E096B0A5-05A8-4892-9B35-83E3C66E252B}">
+      <formula1>"create,update"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47114442-A83F-4F0F-9CDA-49533B7F7997}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>

</xml_diff>